<commit_message>
Major revision of files
</commit_message>
<xml_diff>
--- a/meal dissolved rapid starch.xlsx
+++ b/meal dissolved rapid starch.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A5E9A438-D3D1-4916-BC73-3C6F1B7497F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{891E0A9B-DE0C-41CF-A33A-B1F4DABFF728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meal" sheetId="3" r:id="rId1"/>
@@ -503,7 +503,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -519,8 +519,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -540,7 +539,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="meal"/>
@@ -1140,13 +1139,13 @@
       <c r="B9" s="9">
         <v>1</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9">
         <v>250</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9">
         <v>50</v>
       </c>
       <c r="T9" s="10"/>
@@ -1160,13 +1159,13 @@
       <c r="B10" s="9">
         <v>17</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10">
         <v>50</v>
       </c>
       <c r="T10" s="10"/>
@@ -5720,13 +5719,13 @@
       </c>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A77" s="15">
+      <c r="A77">
         <v>72</v>
       </c>
       <c r="B77" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C77" s="15" t="s">
+      <c r="C77" t="s">
         <v>28</v>
       </c>
       <c r="D77" s="7">
@@ -5735,34 +5734,34 @@
       <c r="E77" s="7">
         <v>0</v>
       </c>
-      <c r="F77" s="15">
-        <v>0</v>
-      </c>
-      <c r="G77" s="15">
-        <v>0</v>
-      </c>
-      <c r="H77" s="16">
-        <v>0</v>
-      </c>
-      <c r="I77" s="15">
-        <v>0</v>
-      </c>
-      <c r="J77" s="15">
-        <v>0</v>
-      </c>
-      <c r="K77" s="15">
-        <v>0</v>
-      </c>
-      <c r="L77" s="15">
-        <v>0</v>
-      </c>
-      <c r="M77" s="15">
-        <v>0</v>
-      </c>
-      <c r="N77" s="15">
-        <v>0</v>
-      </c>
-      <c r="O77" s="15">
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77" s="15">
+        <v>0</v>
+      </c>
+      <c r="I77">
+        <v>0</v>
+      </c>
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+      <c r="L77">
+        <v>0</v>
+      </c>
+      <c r="M77">
+        <v>0</v>
+      </c>
+      <c r="N77">
+        <v>0</v>
+      </c>
+      <c r="O77">
         <v>0</v>
       </c>
       <c r="P77" s="8">
@@ -5788,13 +5787,13 @@
       </c>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A78" s="15">
+      <c r="A78">
         <v>73</v>
       </c>
       <c r="B78" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C78" s="15" t="s">
+      <c r="C78" t="s">
         <v>28</v>
       </c>
       <c r="D78" s="7">
@@ -5803,34 +5802,34 @@
       <c r="E78" s="7">
         <v>0</v>
       </c>
-      <c r="F78" s="15">
-        <v>0</v>
-      </c>
-      <c r="G78" s="15">
-        <v>0</v>
-      </c>
-      <c r="H78" s="16">
-        <v>0</v>
-      </c>
-      <c r="I78" s="15">
-        <v>0</v>
-      </c>
-      <c r="J78" s="15">
-        <v>0</v>
-      </c>
-      <c r="K78" s="15">
-        <v>0</v>
-      </c>
-      <c r="L78" s="15">
-        <v>0</v>
-      </c>
-      <c r="M78" s="15">
-        <v>0</v>
-      </c>
-      <c r="N78" s="15">
-        <v>0</v>
-      </c>
-      <c r="O78" s="15">
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78" s="15">
+        <v>0</v>
+      </c>
+      <c r="I78">
+        <v>0</v>
+      </c>
+      <c r="J78">
+        <v>0</v>
+      </c>
+      <c r="K78">
+        <v>0</v>
+      </c>
+      <c r="L78">
+        <v>0</v>
+      </c>
+      <c r="M78">
+        <v>0</v>
+      </c>
+      <c r="N78">
+        <v>0</v>
+      </c>
+      <c r="O78">
         <v>0</v>
       </c>
       <c r="P78" s="8">
@@ -5856,13 +5855,13 @@
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A79" s="15">
+      <c r="A79">
         <v>74</v>
       </c>
       <c r="B79" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C79" t="s">
         <v>28</v>
       </c>
       <c r="D79" s="7">
@@ -5871,34 +5870,34 @@
       <c r="E79" s="7">
         <v>0</v>
       </c>
-      <c r="F79" s="15">
-        <v>0</v>
-      </c>
-      <c r="G79" s="15">
-        <v>0</v>
-      </c>
-      <c r="H79" s="16">
-        <v>0</v>
-      </c>
-      <c r="I79" s="15">
-        <v>0</v>
-      </c>
-      <c r="J79" s="15">
-        <v>0</v>
-      </c>
-      <c r="K79" s="15">
-        <v>0</v>
-      </c>
-      <c r="L79" s="15">
-        <v>0</v>
-      </c>
-      <c r="M79" s="15">
-        <v>0</v>
-      </c>
-      <c r="N79" s="15">
-        <v>0</v>
-      </c>
-      <c r="O79" s="15">
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79" s="15">
+        <v>0</v>
+      </c>
+      <c r="I79">
+        <v>0</v>
+      </c>
+      <c r="J79">
+        <v>0</v>
+      </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+      <c r="L79">
+        <v>0</v>
+      </c>
+      <c r="M79">
+        <v>0</v>
+      </c>
+      <c r="N79">
+        <v>0</v>
+      </c>
+      <c r="O79">
         <v>0</v>
       </c>
       <c r="P79" s="8">

</xml_diff>

<commit_message>
many update regarding starch digestion and amylase inhibition
</commit_message>
<xml_diff>
--- a/meal dissolved rapid starch.xlsx
+++ b/meal dissolved rapid starch.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{891E0A9B-DE0C-41CF-A33A-B1F4DABFF728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="8_{891E0A9B-DE0C-41CF-A33A-B1F4DABFF728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A8175A7-FA43-46B4-BB8A-44B1AB8528D7}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meal" sheetId="3" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1106" uniqueCount="113">
   <si>
     <t>Inlezen maaltijden</t>
   </si>
@@ -387,6 +387,9 @@
   <si>
     <t>I_a</t>
   </si>
+  <si>
+    <t>citric acid</t>
+  </si>
 </sst>
 </file>
 
@@ -503,7 +506,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -520,6 +523,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -539,7 +544,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="meal"/>
@@ -988,7 +993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y84"/>
+  <dimension ref="A1:X85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="7"/>
@@ -1001,12 +1006,12 @@
     <col min="11" max="16384" width="8.88671875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>76</v>
       </c>
@@ -1017,7 +1022,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>30</v>
       </c>
@@ -1052,9 +1057,8 @@
       <c r="V4" s="8"/>
       <c r="W4" s="8"/>
       <c r="X4" s="8"/>
-      <c r="Y4" s="8"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>27</v>
       </c>
@@ -1072,7 +1076,7 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>0</v>
       </c>
@@ -1092,7 +1096,7 @@
       <c r="U6" s="11"/>
       <c r="V6" s="11"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>1</v>
       </c>
@@ -1112,7 +1116,7 @@
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>300</v>
       </c>
@@ -1132,7 +1136,7 @@
       <c r="U8" s="11"/>
       <c r="V8" s="11"/>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>301</v>
       </c>
@@ -1152,7 +1156,7 @@
       <c r="U9" s="11"/>
       <c r="V9" s="11"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>302</v>
       </c>
@@ -1172,17 +1176,17 @@
       <c r="U10" s="11"/>
       <c r="V10" s="11"/>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>9999</v>
       </c>
       <c r="B11" s="8"/>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
     </row>
-    <row r="13" spans="1:25" s="8" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24" s="8" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="12" t="s">
         <v>72</v>
       </c>
@@ -1250,7 +1254,7 @@
         <v>9999</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>75</v>
       </c>
@@ -1314,7 +1318,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>1</v>
       </c>
@@ -1388,7 +1392,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>42</v>
       </c>
@@ -5565,58 +5569,49 @@
       </c>
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A75" s="7">
-        <v>70</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C75" s="7" t="s">
+      <c r="A75" s="16">
+        <v>68</v>
+      </c>
+      <c r="B75" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="C75" s="16" t="s">
         <v>28</v>
       </c>
       <c r="D75" s="7">
-        <f>water!D60</f>
         <v>0</v>
       </c>
       <c r="E75" s="7">
-        <f>glucose!D60</f>
-        <v>0</v>
-      </c>
-      <c r="F75" s="7">
-        <f>sucrose!D60</f>
-        <v>0</v>
-      </c>
-      <c r="G75" s="7">
-        <f>'milk choc'!D60</f>
-        <v>0</v>
-      </c>
-      <c r="H75" s="13">
-        <f>'milk chocolate arabinose'!D60</f>
-        <v>0</v>
-      </c>
-      <c r="I75" s="7">
-        <f>'gastic milk choc'!D60</f>
-        <v>0</v>
-      </c>
-      <c r="J75" s="7">
-        <f>'gastic milk choc arab'!D60</f>
-        <v>0</v>
-      </c>
-      <c r="K75" s="7">
-        <f>emulsie!D60</f>
-        <v>0</v>
-      </c>
-      <c r="L75" s="7">
-        <f>arabinose!D60</f>
-        <v>0</v>
-      </c>
-      <c r="M75" s="7">
-        <v>0</v>
-      </c>
-      <c r="N75" s="7">
-        <v>0</v>
-      </c>
-      <c r="O75" s="7">
+        <v>0</v>
+      </c>
+      <c r="F75" s="16">
+        <v>0</v>
+      </c>
+      <c r="G75" s="16">
+        <v>0</v>
+      </c>
+      <c r="H75" s="17">
+        <v>0</v>
+      </c>
+      <c r="I75" s="16">
+        <v>0</v>
+      </c>
+      <c r="J75" s="16">
+        <v>0</v>
+      </c>
+      <c r="K75" s="16">
+        <v>0</v>
+      </c>
+      <c r="L75" s="16">
+        <v>0</v>
+      </c>
+      <c r="M75" s="16">
+        <v>0</v>
+      </c>
+      <c r="N75" s="16">
+        <v>0</v>
+      </c>
+      <c r="O75" s="16">
         <v>0</v>
       </c>
       <c r="P75" s="8">
@@ -5643,125 +5638,134 @@
     </row>
     <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76" s="7">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C76" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D76" s="7">
+        <f>water!D60</f>
+        <v>0</v>
+      </c>
+      <c r="E76" s="7">
+        <f>glucose!D60</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="7">
+        <f>sucrose!D60</f>
+        <v>0</v>
+      </c>
+      <c r="G76" s="7">
+        <f>'milk choc'!D60</f>
+        <v>0</v>
+      </c>
+      <c r="H76" s="13">
+        <f>'milk chocolate arabinose'!D60</f>
+        <v>0</v>
+      </c>
+      <c r="I76" s="7">
+        <f>'gastic milk choc'!D60</f>
+        <v>0</v>
+      </c>
+      <c r="J76" s="7">
+        <f>'gastic milk choc arab'!D60</f>
+        <v>0</v>
+      </c>
+      <c r="K76" s="7">
+        <f>emulsie!D60</f>
+        <v>0</v>
+      </c>
+      <c r="L76" s="7">
+        <f>arabinose!D60</f>
+        <v>0</v>
+      </c>
+      <c r="M76" s="7">
+        <v>0</v>
+      </c>
+      <c r="N76" s="7">
+        <v>0</v>
+      </c>
+      <c r="O76" s="7">
+        <v>0</v>
+      </c>
+      <c r="P76" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="8">
+        <v>0</v>
+      </c>
+      <c r="R76" s="8">
+        <v>0</v>
+      </c>
+      <c r="S76" s="8">
+        <v>0</v>
+      </c>
+      <c r="T76" s="8">
+        <v>0</v>
+      </c>
+      <c r="U76" s="8">
+        <v>0</v>
+      </c>
+      <c r="V76" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A77" s="7">
+        <v>71</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D77" s="7">
         <f>water!D61</f>
         <v>0</v>
       </c>
-      <c r="E76" s="7">
+      <c r="E77" s="7">
         <f>glucose!D61</f>
         <v>0</v>
       </c>
-      <c r="F76" s="7">
+      <c r="F77" s="7">
         <f>sucrose!D61</f>
         <v>0</v>
       </c>
-      <c r="G76" s="7">
+      <c r="G77" s="7">
         <f>'milk choc'!D61</f>
         <v>0</v>
       </c>
-      <c r="H76" s="13">
+      <c r="H77" s="13">
         <f>'milk chocolate arabinose'!D61</f>
         <v>0</v>
       </c>
-      <c r="I76" s="7">
+      <c r="I77" s="7">
         <f>'gastic milk choc'!D61</f>
         <v>0</v>
       </c>
-      <c r="J76" s="7">
+      <c r="J77" s="7">
         <f>'gastic milk choc arab'!D61</f>
         <v>0</v>
       </c>
-      <c r="K76" s="7">
+      <c r="K77" s="7">
         <f>emulsie!D61</f>
         <v>0</v>
       </c>
-      <c r="L76" s="7">
+      <c r="L77" s="7">
         <f>arabinose!D61</f>
         <v>0</v>
       </c>
-      <c r="M76" s="7">
-        <v>0</v>
-      </c>
-      <c r="N76" s="7">
-        <v>0</v>
-      </c>
-      <c r="O76" s="7">
-        <v>0</v>
-      </c>
-      <c r="P76" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q76" s="8">
-        <v>0</v>
-      </c>
-      <c r="R76" s="8">
-        <v>0</v>
-      </c>
-      <c r="S76" s="8">
-        <v>0</v>
-      </c>
-      <c r="T76" s="8">
-        <v>0</v>
-      </c>
-      <c r="U76" s="8">
-        <v>0</v>
-      </c>
-      <c r="V76" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>72</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C77" t="s">
-        <v>28</v>
-      </c>
-      <c r="D77" s="7">
-        <v>0</v>
-      </c>
-      <c r="E77" s="7">
-        <v>0</v>
-      </c>
-      <c r="F77">
-        <v>0</v>
-      </c>
-      <c r="G77">
-        <v>0</v>
-      </c>
-      <c r="H77" s="15">
-        <v>0</v>
-      </c>
-      <c r="I77">
-        <v>0</v>
-      </c>
-      <c r="J77">
-        <v>0</v>
-      </c>
-      <c r="K77">
-        <v>0</v>
-      </c>
-      <c r="L77">
-        <v>0</v>
-      </c>
-      <c r="M77">
-        <v>0</v>
-      </c>
-      <c r="N77">
-        <v>0</v>
-      </c>
-      <c r="O77">
+      <c r="M77" s="7">
+        <v>0</v>
+      </c>
+      <c r="N77" s="7">
+        <v>0</v>
+      </c>
+      <c r="O77" s="7">
         <v>0</v>
       </c>
       <c r="P77" s="8">
@@ -5777,7 +5781,7 @@
         <v>0</v>
       </c>
       <c r="T77" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U77" s="8">
         <v>0</v>
@@ -5788,10 +5792,10 @@
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C78" t="s">
         <v>28</v>
@@ -5845,10 +5849,10 @@
         <v>0</v>
       </c>
       <c r="T78" s="8">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U78" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="V78" s="8">
         <v>0</v>
@@ -5856,10 +5860,10 @@
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C79" t="s">
         <v>28</v>
@@ -5916,133 +5920,124 @@
         <v>0</v>
       </c>
       <c r="U79" s="8">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V79" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>74</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C80" t="s">
+        <v>28</v>
+      </c>
+      <c r="D80" s="7">
+        <v>0</v>
+      </c>
+      <c r="E80" s="7">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="G80">
+        <v>0</v>
+      </c>
+      <c r="H80" s="15">
+        <v>0</v>
+      </c>
+      <c r="I80">
+        <v>0</v>
+      </c>
+      <c r="J80">
+        <v>0</v>
+      </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80">
+        <v>0</v>
+      </c>
+      <c r="M80">
+        <v>0</v>
+      </c>
+      <c r="N80">
+        <v>0</v>
+      </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="8">
+        <v>0</v>
+      </c>
+      <c r="R80" s="8">
+        <v>0</v>
+      </c>
+      <c r="S80" s="8">
+        <v>0</v>
+      </c>
+      <c r="T80" s="8">
+        <v>0</v>
+      </c>
+      <c r="U80" s="8">
+        <v>0</v>
+      </c>
+      <c r="V80" s="8">
         <v>100</v>
-      </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A80" s="7">
-        <v>78</v>
-      </c>
-      <c r="B80" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C80" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D80" s="7">
-        <f>water!D62</f>
-        <v>0</v>
-      </c>
-      <c r="E80" s="7">
-        <f>glucose!D62</f>
-        <v>0</v>
-      </c>
-      <c r="F80" s="7">
-        <f>sucrose!D62</f>
-        <v>0</v>
-      </c>
-      <c r="G80" s="7">
-        <f>'milk choc'!D62</f>
-        <v>0</v>
-      </c>
-      <c r="H80" s="13">
-        <f>'milk chocolate arabinose'!D62</f>
-        <v>0</v>
-      </c>
-      <c r="I80" s="7">
-        <f>'gastic milk choc'!D62</f>
-        <v>0</v>
-      </c>
-      <c r="J80" s="7">
-        <f>'gastic milk choc arab'!D62</f>
-        <v>0</v>
-      </c>
-      <c r="K80" s="7">
-        <f>emulsie!D62</f>
-        <v>0</v>
-      </c>
-      <c r="L80" s="7">
-        <f>arabinose!D62</f>
-        <v>0</v>
-      </c>
-      <c r="M80" s="7">
-        <v>0</v>
-      </c>
-      <c r="N80" s="7">
-        <v>0</v>
-      </c>
-      <c r="O80" s="7">
-        <v>0</v>
-      </c>
-      <c r="P80" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q80" s="8">
-        <v>0</v>
-      </c>
-      <c r="R80" s="8">
-        <v>0</v>
-      </c>
-      <c r="S80" s="8">
-        <v>0</v>
-      </c>
-      <c r="T80" s="8">
-        <v>0</v>
-      </c>
-      <c r="U80" s="8">
-        <v>0</v>
-      </c>
-      <c r="V80" s="8">
-        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" s="7">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C81" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D81" s="7">
-        <f>water!D63</f>
+        <f>water!D62</f>
         <v>0</v>
       </c>
       <c r="E81" s="7">
-        <f>glucose!D63</f>
+        <f>glucose!D62</f>
         <v>0</v>
       </c>
       <c r="F81" s="7">
-        <f>sucrose!D63</f>
+        <f>sucrose!D62</f>
         <v>0</v>
       </c>
       <c r="G81" s="7">
-        <f>'milk choc'!D63</f>
+        <f>'milk choc'!D62</f>
         <v>0</v>
       </c>
       <c r="H81" s="13">
-        <f>'milk chocolate arabinose'!D63</f>
+        <f>'milk chocolate arabinose'!D62</f>
         <v>0</v>
       </c>
       <c r="I81" s="7">
-        <f>'gastic milk choc'!D63</f>
+        <f>'gastic milk choc'!D62</f>
         <v>0</v>
       </c>
       <c r="J81" s="7">
-        <f>'gastic milk choc arab'!D63</f>
+        <f>'gastic milk choc arab'!D62</f>
         <v>0</v>
       </c>
       <c r="K81" s="7">
-        <f>emulsie!D63</f>
+        <f>emulsie!D62</f>
         <v>0</v>
       </c>
       <c r="L81" s="7">
-        <f>arabinose!D63</f>
+        <f>arabinose!D62</f>
         <v>0</v>
       </c>
       <c r="M81" s="7">
@@ -6078,48 +6073,48 @@
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82" s="7">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D82" s="7">
-        <f>water!D64</f>
+        <f>water!D63</f>
         <v>0</v>
       </c>
       <c r="E82" s="7">
-        <f>glucose!D64</f>
+        <f>glucose!D63</f>
         <v>0</v>
       </c>
       <c r="F82" s="7">
-        <f>sucrose!D64</f>
+        <f>sucrose!D63</f>
         <v>0</v>
       </c>
       <c r="G82" s="7">
-        <f>'milk choc'!D64</f>
+        <f>'milk choc'!D63</f>
         <v>0</v>
       </c>
       <c r="H82" s="13">
-        <f>'milk chocolate arabinose'!D64</f>
+        <f>'milk chocolate arabinose'!D63</f>
         <v>0</v>
       </c>
       <c r="I82" s="7">
-        <f>'gastic milk choc'!D64</f>
+        <f>'gastic milk choc'!D63</f>
         <v>0</v>
       </c>
       <c r="J82" s="7">
-        <f>'gastic milk choc arab'!D64</f>
+        <f>'gastic milk choc arab'!D63</f>
         <v>0</v>
       </c>
       <c r="K82" s="7">
-        <f>emulsie!D64</f>
+        <f>emulsie!D63</f>
         <v>0</v>
       </c>
       <c r="L82" s="7">
-        <f>arabinose!D64</f>
+        <f>arabinose!D63</f>
         <v>0</v>
       </c>
       <c r="M82" s="7">
@@ -6155,156 +6150,233 @@
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" s="7">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="D83" s="7">
-        <f t="shared" ref="D83:M83" si="0">SUM(D36:D82)</f>
+        <f>water!D64</f>
+        <v>0</v>
+      </c>
+      <c r="E83" s="7">
+        <f>glucose!D64</f>
+        <v>0</v>
+      </c>
+      <c r="F83" s="7">
+        <f>sucrose!D64</f>
+        <v>0</v>
+      </c>
+      <c r="G83" s="7">
+        <f>'milk choc'!D64</f>
+        <v>0</v>
+      </c>
+      <c r="H83" s="13">
+        <f>'milk chocolate arabinose'!D64</f>
+        <v>0</v>
+      </c>
+      <c r="I83" s="7">
+        <f>'gastic milk choc'!D64</f>
+        <v>0</v>
+      </c>
+      <c r="J83" s="7">
+        <f>'gastic milk choc arab'!D64</f>
+        <v>0</v>
+      </c>
+      <c r="K83" s="7">
+        <f>emulsie!D64</f>
+        <v>0</v>
+      </c>
+      <c r="L83" s="7">
+        <f>arabinose!D64</f>
+        <v>0</v>
+      </c>
+      <c r="M83" s="7">
+        <v>0</v>
+      </c>
+      <c r="N83" s="7">
+        <v>0</v>
+      </c>
+      <c r="O83" s="7">
+        <v>0</v>
+      </c>
+      <c r="P83" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="8">
+        <v>0</v>
+      </c>
+      <c r="R83" s="8">
+        <v>0</v>
+      </c>
+      <c r="S83" s="8">
+        <v>0</v>
+      </c>
+      <c r="T83" s="8">
+        <v>0</v>
+      </c>
+      <c r="U83" s="8">
+        <v>0</v>
+      </c>
+      <c r="V83" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A84" s="7">
+        <v>0</v>
+      </c>
+      <c r="D84" s="7">
+        <f t="shared" ref="D84:M84" si="0">SUM(D36:D83)</f>
         <v>100</v>
       </c>
-      <c r="E83" s="7">
+      <c r="E84" s="7">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F83" s="7">
+      <c r="F84" s="7">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="G83" s="7">
+      <c r="G84" s="7">
         <f t="shared" si="0"/>
         <v>100.31</v>
       </c>
-      <c r="H83" s="7">
+      <c r="H84" s="7">
         <f t="shared" si="0"/>
         <v>100.41</v>
       </c>
-      <c r="I83" s="7">
+      <c r="I84" s="7">
         <f t="shared" si="0"/>
         <v>99.83</v>
       </c>
-      <c r="J83" s="7">
+      <c r="J84" s="7">
         <f t="shared" si="0"/>
         <v>99.83</v>
       </c>
-      <c r="K83" s="7">
+      <c r="K84" s="7">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="L83" s="7">
+      <c r="L84" s="7">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M83" s="7">
+      <c r="M84" s="7">
         <f t="shared" si="0"/>
         <v>99</v>
       </c>
-      <c r="N83" s="7">
-        <f t="shared" ref="N83:R83" si="1">SUM(N36:N82)</f>
+      <c r="N84" s="7">
+        <f t="shared" ref="N84:R84" si="1">SUM(N36:N83)</f>
         <v>99</v>
       </c>
-      <c r="O83" s="7">
+      <c r="O84" s="7">
         <f t="shared" si="1"/>
         <v>99</v>
       </c>
-      <c r="P83" s="7">
+      <c r="P84" s="7">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-      <c r="Q83" s="7">
+      <c r="Q84" s="7">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-      <c r="R83" s="7">
+      <c r="R84" s="7">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="S83" s="7">
-        <f t="shared" ref="S83:V83" si="2">SUM(S36:S82)</f>
+      <c r="S84" s="7">
+        <f t="shared" ref="S84:V84" si="2">SUM(S36:S83)</f>
         <v>100</v>
       </c>
-      <c r="T83" s="7">
+      <c r="T84" s="7">
         <f t="shared" si="2"/>
         <v>100</v>
       </c>
-      <c r="U83" s="7">
+      <c r="U84" s="7">
         <f t="shared" si="2"/>
         <v>100</v>
       </c>
-      <c r="V83" s="7">
+      <c r="V84" s="7">
         <f t="shared" si="2"/>
         <v>100</v>
       </c>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B84" s="7" t="s">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="B85" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C84" s="7" t="s">
+      <c r="C85" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D84" s="7">
+      <c r="D85" s="7">
         <f>water!D66</f>
         <v>1</v>
       </c>
-      <c r="E84" s="7">
+      <c r="E85" s="7">
         <f>glucose!D66</f>
         <v>1.44</v>
       </c>
-      <c r="F84" s="7">
+      <c r="F85" s="7">
         <f>sucrose!D66</f>
         <v>1.44</v>
       </c>
-      <c r="G84" s="7">
+      <c r="G85" s="7">
         <f>'milk choc'!D66</f>
         <v>1.3</v>
       </c>
-      <c r="H84" s="13">
+      <c r="H85" s="13">
         <f>'milk chocolate arabinose'!D66</f>
         <v>1.3</v>
       </c>
-      <c r="I84" s="7">
+      <c r="I85" s="7">
         <f>'gastic milk choc'!D66</f>
         <v>1.2</v>
       </c>
-      <c r="J84" s="7">
+      <c r="J85" s="7">
         <f>'gastic milk choc arab'!D66</f>
         <v>1.2</v>
       </c>
-      <c r="K84" s="7">
+      <c r="K85" s="7">
         <f>emulsie!D66</f>
         <v>0.95</v>
       </c>
-      <c r="L84" s="7">
+      <c r="L85" s="7">
         <f>arabinose!D66</f>
         <v>1.44</v>
       </c>
-      <c r="M84" s="7">
+      <c r="M85" s="7">
         <v>1.44</v>
       </c>
-      <c r="N84" s="7">
+      <c r="N85" s="7">
         <v>1.44</v>
       </c>
-      <c r="O84" s="7">
+      <c r="O85" s="7">
         <v>1.44</v>
       </c>
-      <c r="P84" s="8">
+      <c r="P85" s="8">
         <v>1.4</v>
       </c>
-      <c r="Q84" s="8">
+      <c r="Q85" s="8">
         <v>1.4</v>
       </c>
-      <c r="R84" s="8">
+      <c r="R85" s="8">
         <v>1.4</v>
       </c>
-      <c r="S84" s="8">
+      <c r="S85" s="8">
         <v>1.4</v>
       </c>
-      <c r="T84" s="8">
+      <c r="T85" s="8">
         <v>1.4</v>
       </c>
-      <c r="U84" s="8">
+      <c r="U85" s="8">
         <v>1.4</v>
       </c>
-      <c r="V84" s="8">
+      <c r="V85" s="8">
         <v>1.4</v>
       </c>
     </row>

</xml_diff>